<commit_message>
auto: update 0/1 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M271"/>
+  <dimension ref="A1:M273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9664,6 +9664,74 @@
       </c>
       <c r="M271" t="n">
         <v>1.240618</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>03/09</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>1.7589</v>
+      </c>
+      <c r="D272" t="n">
+        <v>1.7589</v>
+      </c>
+      <c r="E272" t="n">
+        <v>0.696948</v>
+      </c>
+      <c r="F272" t="n">
+        <v>0.1199</v>
+      </c>
+      <c r="H272" t="n">
+        <v>0.1199</v>
+      </c>
+      <c r="I272" t="n">
+        <v>1.100305</v>
+      </c>
+      <c r="J272" t="n">
+        <v>0.1325</v>
+      </c>
+      <c r="L272" t="n">
+        <v>0.1325</v>
+      </c>
+      <c r="M272" t="n">
+        <v>1.242262</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>03/10</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>-2.9122</v>
+      </c>
+      <c r="D273" t="n">
+        <v>-2.9122</v>
+      </c>
+      <c r="E273" t="n">
+        <v>0.676652</v>
+      </c>
+      <c r="F273" t="n">
+        <v>0.4692</v>
+      </c>
+      <c r="H273" t="n">
+        <v>0.4692</v>
+      </c>
+      <c r="I273" t="n">
+        <v>1.105468</v>
+      </c>
+      <c r="J273" t="n">
+        <v>0.9009</v>
+      </c>
+      <c r="L273" t="n">
+        <v>0.9009</v>
+      </c>
+      <c r="M273" t="n">
+        <v>1.253454</v>
       </c>
     </row>
   </sheetData>
@@ -9677,7 +9745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E271"/>
+  <dimension ref="A1:E273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14835,6 +14903,44 @@
       </c>
       <c r="E271" t="n">
         <v>1.519301</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>03/09</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>-0.6415999999999999</v>
+      </c>
+      <c r="C272" t="n">
+        <v>-1.6906</v>
+      </c>
+      <c r="D272" t="n">
+        <v>-1.1661</v>
+      </c>
+      <c r="E272" t="n">
+        <v>1.501585</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>03/10</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>3.0406</v>
+      </c>
+      <c r="C273" t="n">
+        <v>2.1616</v>
+      </c>
+      <c r="D273" t="n">
+        <v>2.6011</v>
+      </c>
+      <c r="E273" t="n">
+        <v>1.540643</v>
       </c>
     </row>
   </sheetData>
@@ -14848,7 +14954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E271"/>
+  <dimension ref="A1:E273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20006,6 +20112,44 @@
       </c>
       <c r="E271" t="n">
         <v>1.511215</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>03/09</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>0.4433</v>
+      </c>
+      <c r="C272" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="D272" t="n">
+        <v>1.1533</v>
+      </c>
+      <c r="E272" t="n">
+        <v>1.528645</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>03/10</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>-0.8333</v>
+      </c>
+      <c r="C273" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="D273" t="n">
+        <v>-2.1083</v>
+      </c>
+      <c r="E273" t="n">
+        <v>1.496416</v>
       </c>
     </row>
   </sheetData>
@@ -20019,7 +20163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G251"/>
+  <dimension ref="A1:G253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27309,6 +27453,64 @@
         </is>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>03/09</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>-0.495</v>
+      </c>
+      <c r="C252" t="n">
+        <v>-0.705</v>
+      </c>
+      <c r="D252" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E252" t="n">
+        <v>1.054847</v>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>综合, 美容护理, 社会服务, 纺织服饰, 房地产, 环保</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 有色金属, 机械设备, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>03/10</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="C253" t="n">
+        <v>2.4783</v>
+      </c>
+      <c r="D253" t="n">
+        <v>-1.8583</v>
+      </c>
+      <c r="E253" t="n">
+        <v>1.035245</v>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>综合, 美容护理, 社会服务, 纺织服饰, 房地产, 钢铁</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 有色金属, 机械设备, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update 16/17 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M273"/>
+  <dimension ref="A1:M276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9732,6 +9732,108 @@
       </c>
       <c r="M273" t="n">
         <v>1.253454</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>03/11</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>2.8246</v>
+      </c>
+      <c r="D274" t="n">
+        <v>2.8246</v>
+      </c>
+      <c r="E274" t="n">
+        <v>0.695764</v>
+      </c>
+      <c r="F274" t="n">
+        <v>-0.3685</v>
+      </c>
+      <c r="H274" t="n">
+        <v>-0.3685</v>
+      </c>
+      <c r="I274" t="n">
+        <v>1.101394</v>
+      </c>
+      <c r="J274" t="n">
+        <v>-0.9084</v>
+      </c>
+      <c r="L274" t="n">
+        <v>-0.9084</v>
+      </c>
+      <c r="M274" t="n">
+        <v>1.242067</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>03/12</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>2.4525</v>
+      </c>
+      <c r="D275" t="n">
+        <v>2.4525</v>
+      </c>
+      <c r="E275" t="n">
+        <v>0.712828</v>
+      </c>
+      <c r="F275" t="n">
+        <v>-0.214</v>
+      </c>
+      <c r="H275" t="n">
+        <v>-0.214</v>
+      </c>
+      <c r="I275" t="n">
+        <v>1.099037</v>
+      </c>
+      <c r="J275" t="n">
+        <v>-0.799</v>
+      </c>
+      <c r="L275" t="n">
+        <v>-0.799</v>
+      </c>
+      <c r="M275" t="n">
+        <v>1.232143</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>03/13</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>0.3546</v>
+      </c>
+      <c r="D276" t="n">
+        <v>0.3546</v>
+      </c>
+      <c r="E276" t="n">
+        <v>0.715356</v>
+      </c>
+      <c r="F276" t="n">
+        <v>-0.6158</v>
+      </c>
+      <c r="H276" t="n">
+        <v>-0.6158</v>
+      </c>
+      <c r="I276" t="n">
+        <v>1.09227</v>
+      </c>
+      <c r="J276" t="n">
+        <v>-0.9287</v>
+      </c>
+      <c r="L276" t="n">
+        <v>-0.9287</v>
+      </c>
+      <c r="M276" t="n">
+        <v>1.2207</v>
       </c>
     </row>
   </sheetData>
@@ -9745,7 +9847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E273"/>
+  <dimension ref="A1:E276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14941,6 +15043,63 @@
       </c>
       <c r="E273" t="n">
         <v>1.540643</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>03/11</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>1.3123</v>
+      </c>
+      <c r="C274" t="n">
+        <v>-1.3695</v>
+      </c>
+      <c r="D274" t="n">
+        <v>-0.0286</v>
+      </c>
+      <c r="E274" t="n">
+        <v>1.540202</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>03/12</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>-0.9555</v>
+      </c>
+      <c r="C275" t="n">
+        <v>-1.2442</v>
+      </c>
+      <c r="D275" t="n">
+        <v>-1.0998</v>
+      </c>
+      <c r="E275" t="n">
+        <v>1.523262</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>03/13</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>-0.2184</v>
+      </c>
+      <c r="C276" t="n">
+        <v>-0.7239</v>
+      </c>
+      <c r="D276" t="n">
+        <v>-0.4712</v>
+      </c>
+      <c r="E276" t="n">
+        <v>1.516085</v>
       </c>
     </row>
   </sheetData>
@@ -14954,7 +15113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E273"/>
+  <dimension ref="A1:E276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20150,6 +20309,63 @@
       </c>
       <c r="E273" t="n">
         <v>1.496416</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>03/11</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>0.5867</v>
+      </c>
+      <c r="C274" t="n">
+        <v>-0.235</v>
+      </c>
+      <c r="D274" t="n">
+        <v>0.8217</v>
+      </c>
+      <c r="E274" t="n">
+        <v>1.508711</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>03/12</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>1.3833</v>
+      </c>
+      <c r="C275" t="n">
+        <v>-0.57</v>
+      </c>
+      <c r="D275" t="n">
+        <v>1.9533</v>
+      </c>
+      <c r="E275" t="n">
+        <v>1.538181</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>03/13</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>-1.67</v>
+      </c>
+      <c r="C276" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="D276" t="n">
+        <v>-1.955</v>
+      </c>
+      <c r="E276" t="n">
+        <v>1.50811</v>
       </c>
     </row>
   </sheetData>
@@ -20163,7 +20379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G253"/>
+  <dimension ref="A1:G256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27511,6 +27727,93 @@
         </is>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>03/11</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>-0.4067</v>
+      </c>
+      <c r="C254" t="n">
+        <v>0.1433</v>
+      </c>
+      <c r="D254" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="E254" t="n">
+        <v>1.029551</v>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>综合, 美容护理, 社会服务, 纺织服饰, 房地产, 钢铁</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 有色金属, 机械设备, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>03/12</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>-0.1033</v>
+      </c>
+      <c r="C255" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D255" t="n">
+        <v>0.8967000000000001</v>
+      </c>
+      <c r="E255" t="n">
+        <v>1.038783</v>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>综合, 美容护理, 社会服务, 纺织服饰, 房地产, 钢铁</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 有色金属, 机械设备, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>03/13</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>-0.9817</v>
+      </c>
+      <c r="C256" t="n">
+        <v>-1.515</v>
+      </c>
+      <c r="D256" t="n">
+        <v>0.5333</v>
+      </c>
+      <c r="E256" t="n">
+        <v>1.044323</v>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 房地产, 商贸零售</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 有色金属, 机械设备, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update 19/20 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M277"/>
+  <dimension ref="A1:M278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9868,6 +9868,40 @@
       </c>
       <c r="M277" t="n">
         <v>1.223824</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>03/17</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>1.484</v>
+      </c>
+      <c r="D278" t="n">
+        <v>1.484</v>
+      </c>
+      <c r="E278" t="n">
+        <v>0.71484</v>
+      </c>
+      <c r="F278" t="n">
+        <v>-1.0214</v>
+      </c>
+      <c r="H278" t="n">
+        <v>-1.0214</v>
+      </c>
+      <c r="I278" t="n">
+        <v>1.082196</v>
+      </c>
+      <c r="J278" t="n">
+        <v>-1.7678</v>
+      </c>
+      <c r="L278" t="n">
+        <v>-1.7678</v>
+      </c>
+      <c r="M278" t="n">
+        <v>1.202189</v>
       </c>
     </row>
   </sheetData>
@@ -9881,7 +9915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E277"/>
+  <dimension ref="A1:E278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15153,6 +15187,25 @@
       </c>
       <c r="E277" t="n">
         <v>1.533053</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>03/17</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>-2.2926</v>
+      </c>
+      <c r="C278" t="n">
+        <v>-2.2263</v>
+      </c>
+      <c r="D278" t="n">
+        <v>-2.2595</v>
+      </c>
+      <c r="E278" t="n">
+        <v>1.498415</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: refresh dashboard data to 2026-03-22
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M278"/>
+  <dimension ref="A1:M281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9902,6 +9902,108 @@
       </c>
       <c r="M278" t="n">
         <v>1.202189</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>03/18</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>-1.9583</v>
+      </c>
+      <c r="D279" t="n">
+        <v>-1.9583</v>
+      </c>
+      <c r="E279" t="n">
+        <v>0.700841</v>
+      </c>
+      <c r="F279" t="n">
+        <v>0.5322</v>
+      </c>
+      <c r="H279" t="n">
+        <v>0.5322</v>
+      </c>
+      <c r="I279" t="n">
+        <v>1.087956</v>
+      </c>
+      <c r="J279" t="n">
+        <v>1.1158</v>
+      </c>
+      <c r="L279" t="n">
+        <v>1.1158</v>
+      </c>
+      <c r="M279" t="n">
+        <v>1.215603</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>03/19</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>1.8573</v>
+      </c>
+      <c r="D280" t="n">
+        <v>1.8573</v>
+      </c>
+      <c r="E280" t="n">
+        <v>0.713858</v>
+      </c>
+      <c r="F280" t="n">
+        <v>-0.2331</v>
+      </c>
+      <c r="H280" t="n">
+        <v>-0.2331</v>
+      </c>
+      <c r="I280" t="n">
+        <v>1.08542</v>
+      </c>
+      <c r="J280" t="n">
+        <v>-0.9412</v>
+      </c>
+      <c r="L280" t="n">
+        <v>-0.9412</v>
+      </c>
+      <c r="M280" t="n">
+        <v>1.204162</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>03/20</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>1.0902</v>
+      </c>
+      <c r="D281" t="n">
+        <v>1.0902</v>
+      </c>
+      <c r="E281" t="n">
+        <v>0.721641</v>
+      </c>
+      <c r="F281" t="n">
+        <v>-0.7534</v>
+      </c>
+      <c r="H281" t="n">
+        <v>-0.7534</v>
+      </c>
+      <c r="I281" t="n">
+        <v>1.077242</v>
+      </c>
+      <c r="J281" t="n">
+        <v>-2.2286</v>
+      </c>
+      <c r="L281" t="n">
+        <v>-2.2286</v>
+      </c>
+      <c r="M281" t="n">
+        <v>1.177326</v>
       </c>
     </row>
   </sheetData>
@@ -9915,7 +10017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E278"/>
+  <dimension ref="A1:E281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15206,6 +15308,63 @@
       </c>
       <c r="E278" t="n">
         <v>1.498415</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>03/18</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>2.0215</v>
+      </c>
+      <c r="C279" t="n">
+        <v>1.3605</v>
+      </c>
+      <c r="D279" t="n">
+        <v>1.691</v>
+      </c>
+      <c r="E279" t="n">
+        <v>1.523753</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>03/19</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>-1.1135</v>
+      </c>
+      <c r="C280" t="n">
+        <v>-2.4438</v>
+      </c>
+      <c r="D280" t="n">
+        <v>-1.7786</v>
+      </c>
+      <c r="E280" t="n">
+        <v>1.496651</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>03/20</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>1.2994</v>
+      </c>
+      <c r="C281" t="n">
+        <v>-1.5479</v>
+      </c>
+      <c r="D281" t="n">
+        <v>-0.1242</v>
+      </c>
+      <c r="E281" t="n">
+        <v>1.494791</v>
       </c>
     </row>
   </sheetData>
@@ -15219,7 +15378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E278"/>
+  <dimension ref="A1:E281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20510,6 +20669,63 @@
       </c>
       <c r="E278" t="n">
         <v>1.428355</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>03/18</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>-0.6233</v>
+      </c>
+      <c r="C279" t="n">
+        <v>-0.155</v>
+      </c>
+      <c r="D279" t="n">
+        <v>-0.4683</v>
+      </c>
+      <c r="E279" t="n">
+        <v>1.421665</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>03/19</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>-2.7867</v>
+      </c>
+      <c r="C280" t="n">
+        <v>-1.575</v>
+      </c>
+      <c r="D280" t="n">
+        <v>-1.2117</v>
+      </c>
+      <c r="E280" t="n">
+        <v>1.404439</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>03/20</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>-1.1033</v>
+      </c>
+      <c r="C281" t="n">
+        <v>-1.255</v>
+      </c>
+      <c r="D281" t="n">
+        <v>0.1517</v>
+      </c>
+      <c r="E281" t="n">
+        <v>1.406569</v>
       </c>
     </row>
   </sheetData>
@@ -20523,7 +20739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G258"/>
+  <dimension ref="A1:G261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28016,6 +28232,93 @@
         </is>
       </c>
     </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>03/18</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>0.3433</v>
+      </c>
+      <c r="C259" t="n">
+        <v>1.8483</v>
+      </c>
+      <c r="D259" t="n">
+        <v>-1.505</v>
+      </c>
+      <c r="E259" t="n">
+        <v>1.052995</v>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 房地产, 商贸零售</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 有色金属, 机械设备, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>03/19</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>-2.435</v>
+      </c>
+      <c r="C260" t="n">
+        <v>-2.565</v>
+      </c>
+      <c r="D260" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E260" t="n">
+        <v>1.054364</v>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 房地产, 商贸零售</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 有色金属, 机械设备, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>03/20</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>-2.6167</v>
+      </c>
+      <c r="C261" t="n">
+        <v>-0.8917</v>
+      </c>
+      <c r="D261" t="n">
+        <v>-1.725</v>
+      </c>
+      <c r="E261" t="n">
+        <v>1.036177</v>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 房地产</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 有色金属, 机械设备, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update 20/22 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M281"/>
+  <dimension ref="A1:M285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10004,6 +10004,142 @@
       </c>
       <c r="M281" t="n">
         <v>1.177326</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>03/23</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>1.7755</v>
+      </c>
+      <c r="D282" t="n">
+        <v>1.7755</v>
+      </c>
+      <c r="E282" t="n">
+        <v>0.734453</v>
+      </c>
+      <c r="F282" t="n">
+        <v>-0.9802</v>
+      </c>
+      <c r="H282" t="n">
+        <v>-0.9802</v>
+      </c>
+      <c r="I282" t="n">
+        <v>1.066683</v>
+      </c>
+      <c r="J282" t="n">
+        <v>-2.1259</v>
+      </c>
+      <c r="L282" t="n">
+        <v>-2.1259</v>
+      </c>
+      <c r="M282" t="n">
+        <v>1.152297</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>03/24</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>-0.7865</v>
+      </c>
+      <c r="D283" t="n">
+        <v>-0.7865</v>
+      </c>
+      <c r="E283" t="n">
+        <v>0.728677</v>
+      </c>
+      <c r="F283" t="n">
+        <v>0.8482</v>
+      </c>
+      <c r="H283" t="n">
+        <v>0.8482</v>
+      </c>
+      <c r="I283" t="n">
+        <v>1.075731</v>
+      </c>
+      <c r="J283" t="n">
+        <v>2.4572</v>
+      </c>
+      <c r="L283" t="n">
+        <v>2.4572</v>
+      </c>
+      <c r="M283" t="n">
+        <v>1.180612</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>03/25</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>-1.6624</v>
+      </c>
+      <c r="D284" t="n">
+        <v>-1.6624</v>
+      </c>
+      <c r="E284" t="n">
+        <v>0.7165629999999999</v>
+      </c>
+      <c r="F284" t="n">
+        <v>0.3427</v>
+      </c>
+      <c r="H284" t="n">
+        <v>0.3427</v>
+      </c>
+      <c r="I284" t="n">
+        <v>1.079417</v>
+      </c>
+      <c r="J284" t="n">
+        <v>0.8823</v>
+      </c>
+      <c r="L284" t="n">
+        <v>0.8823</v>
+      </c>
+      <c r="M284" t="n">
+        <v>1.191028</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>2.0672</v>
+      </c>
+      <c r="D285" t="n">
+        <v>2.0672</v>
+      </c>
+      <c r="E285" t="n">
+        <v>0.731376</v>
+      </c>
+      <c r="F285" t="n">
+        <v>-0.0925</v>
+      </c>
+      <c r="H285" t="n">
+        <v>-0.0925</v>
+      </c>
+      <c r="I285" t="n">
+        <v>1.078419</v>
+      </c>
+      <c r="J285" t="n">
+        <v>-0.2593</v>
+      </c>
+      <c r="L285" t="n">
+        <v>-0.2593</v>
+      </c>
+      <c r="M285" t="n">
+        <v>1.18794</v>
       </c>
     </row>
   </sheetData>
@@ -10017,7 +10153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E281"/>
+  <dimension ref="A1:E285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15365,6 +15501,82 @@
       </c>
       <c r="E281" t="n">
         <v>1.494791</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>03/23</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>-3.4868</v>
+      </c>
+      <c r="C282" t="n">
+        <v>-4.3138</v>
+      </c>
+      <c r="D282" t="n">
+        <v>-3.9003</v>
+      </c>
+      <c r="E282" t="n">
+        <v>1.43649</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>03/24</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>0.5046</v>
+      </c>
+      <c r="C283" t="n">
+        <v>2.327</v>
+      </c>
+      <c r="D283" t="n">
+        <v>1.4158</v>
+      </c>
+      <c r="E283" t="n">
+        <v>1.456827</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>03/25</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>2.0122</v>
+      </c>
+      <c r="C284" t="n">
+        <v>1.9074</v>
+      </c>
+      <c r="D284" t="n">
+        <v>1.9598</v>
+      </c>
+      <c r="E284" t="n">
+        <v>1.485378</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>-1.3411</v>
+      </c>
+      <c r="C285" t="n">
+        <v>-2.0226</v>
+      </c>
+      <c r="D285" t="n">
+        <v>-1.6819</v>
+      </c>
+      <c r="E285" t="n">
+        <v>1.460397</v>
       </c>
     </row>
   </sheetData>
@@ -15378,7 +15590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E281"/>
+  <dimension ref="A1:E285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20726,6 +20938,82 @@
       </c>
       <c r="E281" t="n">
         <v>1.406569</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>03/23</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>-2.92</v>
+      </c>
+      <c r="C282" t="n">
+        <v>-4.04</v>
+      </c>
+      <c r="D282" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="E282" t="n">
+        <v>1.422323</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>03/24</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>2.1067</v>
+      </c>
+      <c r="C283" t="n">
+        <v>2.075</v>
+      </c>
+      <c r="D283" t="n">
+        <v>0.0317</v>
+      </c>
+      <c r="E283" t="n">
+        <v>1.422773</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>03/25</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>1.1667</v>
+      </c>
+      <c r="C284" t="n">
+        <v>0.825</v>
+      </c>
+      <c r="D284" t="n">
+        <v>0.3417</v>
+      </c>
+      <c r="E284" t="n">
+        <v>1.427635</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>-0.9467</v>
+      </c>
+      <c r="C285" t="n">
+        <v>-1.015</v>
+      </c>
+      <c r="D285" t="n">
+        <v>0.0683</v>
+      </c>
+      <c r="E285" t="n">
+        <v>1.42861</v>
       </c>
     </row>
   </sheetData>
@@ -20739,7 +21027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G261"/>
+  <dimension ref="A1:G265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28319,6 +28607,122 @@
         </is>
       </c>
     </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>03/23</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>-5.5467</v>
+      </c>
+      <c r="C262" t="n">
+        <v>-4.4883</v>
+      </c>
+      <c r="D262" t="n">
+        <v>-1.0583</v>
+      </c>
+      <c r="E262" t="n">
+        <v>1.02521</v>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 房地产</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 机械设备, 有色金属, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>03/24</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>2.8433</v>
+      </c>
+      <c r="C263" t="n">
+        <v>2.3183</v>
+      </c>
+      <c r="D263" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="E263" t="n">
+        <v>1.030593</v>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 房地产</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 机械设备, 有色金属, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>03/25</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>2.2433</v>
+      </c>
+      <c r="C264" t="n">
+        <v>2.4317</v>
+      </c>
+      <c r="D264" t="n">
+        <v>-0.1883</v>
+      </c>
+      <c r="E264" t="n">
+        <v>1.028652</v>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 房地产</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 有色金属, 机械设备, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>-1.4167</v>
+      </c>
+      <c r="C265" t="n">
+        <v>-1.9533</v>
+      </c>
+      <c r="D265" t="n">
+        <v>0.5367</v>
+      </c>
+      <c r="E265" t="n">
+        <v>1.034172</v>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 房地产</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 机械设备, 有色金属, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update 21/22 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -15643,7 +15643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E285"/>
+  <dimension ref="A1:E286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21067,6 +21067,25 @@
       </c>
       <c r="E285" t="n">
         <v>1.42861</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>03/27</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="C286" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="D286" t="n">
+        <v>-1.21</v>
+      </c>
+      <c r="E286" t="n">
+        <v>1.411324</v>
       </c>
     </row>
   </sheetData>
@@ -21080,7 +21099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G265"/>
+  <dimension ref="A1:G266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28776,6 +28795,35 @@
         </is>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>03/27</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>1.1133</v>
+      </c>
+      <c r="C266" t="n">
+        <v>1.0433</v>
+      </c>
+      <c r="D266" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E266" t="n">
+        <v>1.034896</v>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 房地产</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 机械设备, 有色金属, 计算机, 通信</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update 17/22 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M287"/>
+  <dimension ref="A1:M288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10208,6 +10208,40 @@
       </c>
       <c r="M287" t="n">
         <v>1.207128</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>03/31</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>1.4262</v>
+      </c>
+      <c r="D288" t="n">
+        <v>1.4262</v>
+      </c>
+      <c r="E288" t="n">
+        <v>0.749651</v>
+      </c>
+      <c r="F288" t="n">
+        <v>-0.3548</v>
+      </c>
+      <c r="H288" t="n">
+        <v>-0.3548</v>
+      </c>
+      <c r="I288" t="n">
+        <v>1.08202</v>
+      </c>
+      <c r="J288" t="n">
+        <v>-0.7337</v>
+      </c>
+      <c r="L288" t="n">
+        <v>-0.7337</v>
+      </c>
+      <c r="M288" t="n">
+        <v>1.198271</v>
       </c>
     </row>
   </sheetData>
@@ -10221,7 +10255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E287"/>
+  <dimension ref="A1:E288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15683,6 +15717,25 @@
       </c>
       <c r="E287" t="n">
         <v>1.461143</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>03/31</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>-2.7007</v>
+      </c>
+      <c r="C288" t="n">
+        <v>-2.5937</v>
+      </c>
+      <c r="D288" t="n">
+        <v>-2.6472</v>
+      </c>
+      <c r="E288" t="n">
+        <v>1.422463</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update 20/21 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M288"/>
+  <dimension ref="A1:M289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10242,6 +10242,40 @@
       </c>
       <c r="M288" t="n">
         <v>1.198271</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>04/01</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>-3.2734</v>
+      </c>
+      <c r="D289" t="n">
+        <v>-3.2734</v>
+      </c>
+      <c r="E289" t="n">
+        <v>0.725111</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0.3923</v>
+      </c>
+      <c r="H289" t="n">
+        <v>0.3923</v>
+      </c>
+      <c r="I289" t="n">
+        <v>1.086265</v>
+      </c>
+      <c r="J289" t="n">
+        <v>0.3529</v>
+      </c>
+      <c r="L289" t="n">
+        <v>0.3529</v>
+      </c>
+      <c r="M289" t="n">
+        <v>1.2025</v>
       </c>
     </row>
   </sheetData>
@@ -10255,7 +10289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E288"/>
+  <dimension ref="A1:E289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15736,6 +15770,25 @@
       </c>
       <c r="E288" t="n">
         <v>1.422463</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>04/01</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>1.9646</v>
+      </c>
+      <c r="C289" t="n">
+        <v>3.3328</v>
+      </c>
+      <c r="D289" t="n">
+        <v>2.6487</v>
+      </c>
+      <c r="E289" t="n">
+        <v>1.46014</v>
       </c>
     </row>
   </sheetData>
@@ -15749,7 +15802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E287"/>
+  <dimension ref="A1:E288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21211,6 +21264,25 @@
       </c>
       <c r="E287" t="n">
         <v>1.412194</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>03/31</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>-2.2933</v>
+      </c>
+      <c r="C288" t="n">
+        <v>-0.08500000000000001</v>
+      </c>
+      <c r="D288" t="n">
+        <v>-2.2083</v>
+      </c>
+      <c r="E288" t="n">
+        <v>1.381008</v>
       </c>
     </row>
   </sheetData>
@@ -21224,7 +21296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G267"/>
+  <dimension ref="A1:G268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28978,6 +29050,35 @@
         </is>
       </c>
     </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>03/31</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="C268" t="n">
+        <v>-1.9967</v>
+      </c>
+      <c r="D268" t="n">
+        <v>1.0367</v>
+      </c>
+      <c r="E268" t="n">
+        <v>1.04613</v>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 房地产</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 机械设备, 有色金属, 通信, 计算机</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update 18/22 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -15961,7 +15961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E291"/>
+  <dimension ref="A1:E292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21499,6 +21499,25 @@
       </c>
       <c r="E291" t="n">
         <v>1.354919</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>04/07</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>1.3033</v>
+      </c>
+      <c r="C292" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="D292" t="n">
+        <v>1.4733</v>
+      </c>
+      <c r="E292" t="n">
+        <v>1.374881</v>
       </c>
     </row>
   </sheetData>
@@ -21512,7 +21531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G271"/>
+  <dimension ref="A1:G272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29382,6 +29401,35 @@
         </is>
       </c>
     </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>04/07</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>0.8183</v>
+      </c>
+      <c r="C272" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D272" t="n">
+        <v>0.3283</v>
+      </c>
+      <c r="E272" t="n">
+        <v>1.030806</v>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 房地产</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 计算机, 有色金属</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update 3/3 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M292"/>
+  <dimension ref="A1:M293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10378,6 +10378,40 @@
       </c>
       <c r="M292" t="n">
         <v>1.195693</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>04/08</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>-5.3712</v>
+      </c>
+      <c r="D293" t="n">
+        <v>-5.3712</v>
+      </c>
+      <c r="E293" t="n">
+        <v>0.692064</v>
+      </c>
+      <c r="F293" t="n">
+        <v>0.5855</v>
+      </c>
+      <c r="H293" t="n">
+        <v>0.5855</v>
+      </c>
+      <c r="I293" t="n">
+        <v>1.091831</v>
+      </c>
+      <c r="J293" t="n">
+        <v>0.9177999999999999</v>
+      </c>
+      <c r="L293" t="n">
+        <v>0.9177999999999999</v>
+      </c>
+      <c r="M293" t="n">
+        <v>1.206667</v>
       </c>
     </row>
   </sheetData>
@@ -10391,7 +10425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E292"/>
+  <dimension ref="A1:E293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15948,6 +15982,25 @@
       </c>
       <c r="E292" t="n">
         <v>1.427059</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>04/08</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>5.9097</v>
+      </c>
+      <c r="C293" t="n">
+        <v>6.1754</v>
+      </c>
+      <c r="D293" t="n">
+        <v>6.0426</v>
+      </c>
+      <c r="E293" t="n">
+        <v>1.51329</v>
       </c>
     </row>
   </sheetData>
@@ -15961,7 +16014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E291"/>
+  <dimension ref="A1:E293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21499,6 +21552,44 @@
       </c>
       <c r="E291" t="n">
         <v>1.354919</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>04/07</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>1.3033</v>
+      </c>
+      <c r="C292" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="D292" t="n">
+        <v>1.4733</v>
+      </c>
+      <c r="E292" t="n">
+        <v>1.374881</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>04/08</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="C293" t="n">
+        <v>1.665</v>
+      </c>
+      <c r="D293" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="E293" t="n">
+        <v>1.387324</v>
       </c>
     </row>
   </sheetData>
@@ -21512,7 +21603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G271"/>
+  <dimension ref="A1:G273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29382,6 +29473,64 @@
         </is>
       </c>
     </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>04/07</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>0.8183</v>
+      </c>
+      <c r="C272" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D272" t="n">
+        <v>0.3283</v>
+      </c>
+      <c r="E272" t="n">
+        <v>1.030806</v>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 房地产</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 计算机, 有色金属</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>04/08</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>3.335</v>
+      </c>
+      <c r="C273" t="n">
+        <v>5.1917</v>
+      </c>
+      <c r="D273" t="n">
+        <v>-1.8567</v>
+      </c>
+      <c r="E273" t="n">
+        <v>1.011668</v>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 钢铁</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 基础化工</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update 18/21 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -16014,7 +16014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E292"/>
+  <dimension ref="A1:E293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21571,6 +21571,25 @@
       </c>
       <c r="E292" t="n">
         <v>1.374881</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>04/08</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="C293" t="n">
+        <v>1.665</v>
+      </c>
+      <c r="D293" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="E293" t="n">
+        <v>1.387324</v>
       </c>
     </row>
   </sheetData>
@@ -21584,7 +21603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G272"/>
+  <dimension ref="A1:G273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29483,6 +29502,35 @@
         </is>
       </c>
     </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>04/08</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>3.335</v>
+      </c>
+      <c r="C273" t="n">
+        <v>5.1917</v>
+      </c>
+      <c r="D273" t="n">
+        <v>-1.8567</v>
+      </c>
+      <c r="E273" t="n">
+        <v>1.011668</v>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 商贸零售, 钢铁</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 基础化工</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update am 17/21 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M295"/>
+  <dimension ref="A1:M296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10480,6 +10480,40 @@
       </c>
       <c r="M295" t="n">
         <v>1.195263</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>04/13</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>-0.869</v>
+      </c>
+      <c r="D296" t="n">
+        <v>-0.869</v>
+      </c>
+      <c r="E296" t="n">
+        <v>0.676287</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="H296" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="I296" t="n">
+        <v>1.090283</v>
+      </c>
+      <c r="J296" t="n">
+        <v>0.0973</v>
+      </c>
+      <c r="L296" t="n">
+        <v>0.0973</v>
+      </c>
+      <c r="M296" t="n">
+        <v>1.196426</v>
       </c>
     </row>
   </sheetData>
@@ -10493,7 +10527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E295"/>
+  <dimension ref="A1:E296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16107,6 +16141,25 @@
       </c>
       <c r="E295" t="n">
         <v>1.542769</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>04/13</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>0.8018</v>
+      </c>
+      <c r="C296" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="D296" t="n">
+        <v>0.7964</v>
+      </c>
+      <c r="E296" t="n">
+        <v>1.555056</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update pm 22/23 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M295"/>
+  <dimension ref="A1:M296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10480,6 +10480,40 @@
       </c>
       <c r="M295" t="n">
         <v>1.195263</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>04/13</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>-0.869</v>
+      </c>
+      <c r="D296" t="n">
+        <v>-0.869</v>
+      </c>
+      <c r="E296" t="n">
+        <v>0.676287</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="H296" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="I296" t="n">
+        <v>1.090283</v>
+      </c>
+      <c r="J296" t="n">
+        <v>0.0973</v>
+      </c>
+      <c r="L296" t="n">
+        <v>0.0973</v>
+      </c>
+      <c r="M296" t="n">
+        <v>1.196426</v>
       </c>
     </row>
   </sheetData>
@@ -10493,7 +10527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E295"/>
+  <dimension ref="A1:E296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16107,6 +16141,25 @@
       </c>
       <c r="E295" t="n">
         <v>1.542769</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>04/13</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>0.8018</v>
+      </c>
+      <c r="C296" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="D296" t="n">
+        <v>0.7964</v>
+      </c>
+      <c r="E296" t="n">
+        <v>1.555056</v>
       </c>
     </row>
   </sheetData>
@@ -16120,7 +16173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E295"/>
+  <dimension ref="A1:E296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21734,6 +21787,25 @@
       </c>
       <c r="E295" t="n">
         <v>1.391621</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>04/13</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>0.6933</v>
+      </c>
+      <c r="C296" t="n">
+        <v>-0.72</v>
+      </c>
+      <c r="D296" t="n">
+        <v>1.4133</v>
+      </c>
+      <c r="E296" t="n">
+        <v>1.411289</v>
       </c>
     </row>
   </sheetData>
@@ -21747,7 +21819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G275"/>
+  <dimension ref="A1:G276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29733,6 +29805,35 @@
         </is>
       </c>
     </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>04/13</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="C276" t="n">
+        <v>0.5017</v>
+      </c>
+      <c r="D276" t="n">
+        <v>-0.3567</v>
+      </c>
+      <c r="E276" t="n">
+        <v>0.981508</v>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 钢铁, 商贸零售</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 基础化工</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update am 18/22 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M296"/>
+  <dimension ref="A1:M297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10514,6 +10514,40 @@
       </c>
       <c r="M296" t="n">
         <v>1.196426</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>04/14</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>-1.9522</v>
+      </c>
+      <c r="D297" t="n">
+        <v>-1.9522</v>
+      </c>
+      <c r="E297" t="n">
+        <v>0.663084</v>
+      </c>
+      <c r="F297" t="n">
+        <v>0.0886</v>
+      </c>
+      <c r="H297" t="n">
+        <v>0.0886</v>
+      </c>
+      <c r="I297" t="n">
+        <v>1.091249</v>
+      </c>
+      <c r="J297" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="L297" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="M297" t="n">
+        <v>1.197514</v>
       </c>
     </row>
   </sheetData>
@@ -10527,7 +10561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E296"/>
+  <dimension ref="A1:E297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16160,6 +16194,25 @@
       </c>
       <c r="E296" t="n">
         <v>1.555056</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>04/14</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>2.3613</v>
+      </c>
+      <c r="C297" t="n">
+        <v>2.1657</v>
+      </c>
+      <c r="D297" t="n">
+        <v>2.2635</v>
+      </c>
+      <c r="E297" t="n">
+        <v>1.590254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update am 21/22 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -16438,7 +16438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E300"/>
+  <dimension ref="A1:E301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22147,6 +22147,25 @@
       </c>
       <c r="E300" t="n">
         <v>1.429376</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>04/20</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>-0.0267</v>
+      </c>
+      <c r="C301" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="D301" t="n">
+        <v>-0.1817</v>
+      </c>
+      <c r="E301" t="n">
+        <v>1.42678</v>
       </c>
     </row>
   </sheetData>
@@ -22160,7 +22179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G280"/>
+  <dimension ref="A1:G281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30291,6 +30310,35 @@
         </is>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>04/20</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>0.3017</v>
+      </c>
+      <c r="C281" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="D281" t="n">
+        <v>-0.5033</v>
+      </c>
+      <c r="E281" t="n">
+        <v>0.95028</v>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 纺织服饰, 社会服务, 钢铁, 商贸零售</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 计算机</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update pm 23/24 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M302"/>
+  <dimension ref="A1:M303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10718,6 +10718,40 @@
       </c>
       <c r="M302" t="n">
         <v>1.21255</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>04/22</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>-1.7227</v>
+      </c>
+      <c r="D303" t="n">
+        <v>-1.7227</v>
+      </c>
+      <c r="E303" t="n">
+        <v>0.647161</v>
+      </c>
+      <c r="F303" t="n">
+        <v>0.4165</v>
+      </c>
+      <c r="H303" t="n">
+        <v>0.4165</v>
+      </c>
+      <c r="I303" t="n">
+        <v>1.106411</v>
+      </c>
+      <c r="J303" t="n">
+        <v>0.1463</v>
+      </c>
+      <c r="L303" t="n">
+        <v>0.1463</v>
+      </c>
+      <c r="M303" t="n">
+        <v>1.214324</v>
       </c>
     </row>
   </sheetData>
@@ -10731,7 +10765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E302"/>
+  <dimension ref="A1:E303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16478,6 +16512,25 @@
       </c>
       <c r="E302" t="n">
         <v>1.63184</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>04/22</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>1.7301</v>
+      </c>
+      <c r="C303" t="n">
+        <v>1.7146</v>
+      </c>
+      <c r="D303" t="n">
+        <v>1.7224</v>
+      </c>
+      <c r="E303" t="n">
+        <v>1.659946</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update am 20/22 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -16650,7 +16650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E304"/>
+  <dimension ref="A1:E305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22435,6 +22435,25 @@
       </c>
       <c r="E304" t="n">
         <v>1.430101</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>04/24</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="C305" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="D305" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="E305" t="n">
+        <v>1.427241</v>
       </c>
     </row>
   </sheetData>
@@ -22448,7 +22467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G284"/>
+  <dimension ref="A1:G285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30695,6 +30714,35 @@
         </is>
       </c>
     </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>04/24</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>-0.3233</v>
+      </c>
+      <c r="C285" t="n">
+        <v>-0.655</v>
+      </c>
+      <c r="D285" t="n">
+        <v>0.3317</v>
+      </c>
+      <c r="E285" t="n">
+        <v>0.948219</v>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 纺织服饰, 社会服务, 钢铁, 煤炭</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 计算机</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update am 18/23 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M305"/>
+  <dimension ref="A1:M306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10820,6 +10820,40 @@
       </c>
       <c r="M305" t="n">
         <v>1.193469</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>04/27</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>-3.9786</v>
+      </c>
+      <c r="D306" t="n">
+        <v>-3.9786</v>
+      </c>
+      <c r="E306" t="n">
+        <v>0.622624</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0.0796</v>
+      </c>
+      <c r="H306" t="n">
+        <v>0.0796</v>
+      </c>
+      <c r="I306" t="n">
+        <v>1.096841</v>
+      </c>
+      <c r="J306" t="n">
+        <v>0.9751</v>
+      </c>
+      <c r="L306" t="n">
+        <v>0.9751</v>
+      </c>
+      <c r="M306" t="n">
+        <v>1.205106</v>
       </c>
     </row>
   </sheetData>
@@ -10833,7 +10867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E305"/>
+  <dimension ref="A1:E306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16637,6 +16671,25 @@
       </c>
       <c r="E305" t="n">
         <v>1.642659</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>04/27</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>-0.5179</v>
+      </c>
+      <c r="C306" t="n">
+        <v>3.7628</v>
+      </c>
+      <c r="D306" t="n">
+        <v>1.6224</v>
+      </c>
+      <c r="E306" t="n">
+        <v>1.66931</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update am 21/23 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M305"/>
+  <dimension ref="A1:M306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10820,6 +10820,40 @@
       </c>
       <c r="M305" t="n">
         <v>1.193469</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>04/27</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>-3.9786</v>
+      </c>
+      <c r="D306" t="n">
+        <v>-3.9786</v>
+      </c>
+      <c r="E306" t="n">
+        <v>0.622624</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0.0796</v>
+      </c>
+      <c r="H306" t="n">
+        <v>0.0796</v>
+      </c>
+      <c r="I306" t="n">
+        <v>1.096841</v>
+      </c>
+      <c r="J306" t="n">
+        <v>0.9751</v>
+      </c>
+      <c r="L306" t="n">
+        <v>0.9751</v>
+      </c>
+      <c r="M306" t="n">
+        <v>1.205106</v>
       </c>
     </row>
   </sheetData>
@@ -10833,7 +10867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E305"/>
+  <dimension ref="A1:E306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16637,6 +16671,25 @@
       </c>
       <c r="E305" t="n">
         <v>1.642659</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>04/27</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>-0.5179</v>
+      </c>
+      <c r="C306" t="n">
+        <v>3.7628</v>
+      </c>
+      <c r="D306" t="n">
+        <v>1.6224</v>
+      </c>
+      <c r="E306" t="n">
+        <v>1.66931</v>
       </c>
     </row>
   </sheetData>
@@ -16650,7 +16703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E305"/>
+  <dimension ref="A1:E306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22454,6 +22507,25 @@
       </c>
       <c r="E305" t="n">
         <v>1.427241</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>04/27</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="C306" t="n">
+        <v>-1.01</v>
+      </c>
+      <c r="D306" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E306" t="n">
+        <v>1.431523</v>
       </c>
     </row>
   </sheetData>
@@ -22467,7 +22539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G285"/>
+  <dimension ref="A1:G286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30743,6 +30815,35 @@
         </is>
       </c>
     </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>04/27</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>0.3783</v>
+      </c>
+      <c r="C286" t="n">
+        <v>0.5217000000000001</v>
+      </c>
+      <c r="D286" t="n">
+        <v>-0.1433</v>
+      </c>
+      <c r="E286" t="n">
+        <v>0.946859</v>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 纺织服饰, 社会服务, 钢铁, 煤炭</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 计算机</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update am 17/23 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M307"/>
+  <dimension ref="A1:M308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10888,6 +10888,40 @@
       </c>
       <c r="M307" t="n">
         <v>1.1943</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>04/29</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D308" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E308" t="n">
+        <v>0.641773</v>
+      </c>
+      <c r="F308" t="n">
+        <v>-0.0658</v>
+      </c>
+      <c r="H308" t="n">
+        <v>-0.0658</v>
+      </c>
+      <c r="I308" t="n">
+        <v>1.090014</v>
+      </c>
+      <c r="J308" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="L308" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="M308" t="n">
+        <v>1.195482</v>
       </c>
     </row>
   </sheetData>
@@ -10901,7 +10935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E307"/>
+  <dimension ref="A1:E308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16743,6 +16777,25 @@
       </c>
       <c r="E307" t="n">
         <v>1.646484</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>04/29</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>2.515</v>
+      </c>
+      <c r="C308" t="n">
+        <v>0.3254</v>
+      </c>
+      <c r="D308" t="n">
+        <v>1.4202</v>
+      </c>
+      <c r="E308" t="n">
+        <v>1.669868</v>
       </c>
     </row>
   </sheetData>
@@ -16756,7 +16809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E307"/>
+  <dimension ref="A1:E308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22598,6 +22651,25 @@
       </c>
       <c r="E307" t="n">
         <v>1.429781</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>04/29</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>2.5167</v>
+      </c>
+      <c r="C308" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="D308" t="n">
+        <v>1.8617</v>
+      </c>
+      <c r="E308" t="n">
+        <v>1.456399</v>
       </c>
     </row>
   </sheetData>
@@ -22611,7 +22683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G287"/>
+  <dimension ref="A1:G288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30945,6 +31017,35 @@
         </is>
       </c>
     </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>04/29</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>1.415</v>
+      </c>
+      <c r="C288" t="n">
+        <v>1.8283</v>
+      </c>
+      <c r="D288" t="n">
+        <v>-0.4133</v>
+      </c>
+      <c r="E288" t="n">
+        <v>0.961019</v>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 纺织服饰, 社会服务, 煤炭, 钢铁</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 计算机</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update am 22/25 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M309"/>
+  <dimension ref="A1:M310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10956,6 +10956,40 @@
       </c>
       <c r="M309" t="n">
         <v>1.202452</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>05/06</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>-5.1806</v>
+      </c>
+      <c r="D310" t="n">
+        <v>-5.1806</v>
+      </c>
+      <c r="E310" t="n">
+        <v>0.5749379999999999</v>
+      </c>
+      <c r="F310" t="n">
+        <v>0.387</v>
+      </c>
+      <c r="H310" t="n">
+        <v>0.387</v>
+      </c>
+      <c r="I310" t="n">
+        <v>1.097828</v>
+      </c>
+      <c r="J310" t="n">
+        <v>0.5800999999999999</v>
+      </c>
+      <c r="L310" t="n">
+        <v>0.5800999999999999</v>
+      </c>
+      <c r="M310" t="n">
+        <v>1.209428</v>
       </c>
     </row>
   </sheetData>
@@ -10969,7 +11003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E309"/>
+  <dimension ref="A1:E310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16849,6 +16883,25 @@
       </c>
       <c r="E309" t="n">
         <v>1.710959</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>05/06</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>2.747</v>
+      </c>
+      <c r="C310" t="n">
+        <v>5.4664</v>
+      </c>
+      <c r="D310" t="n">
+        <v>4.1067</v>
+      </c>
+      <c r="E310" t="n">
+        <v>1.781223</v>
       </c>
     </row>
   </sheetData>
@@ -16862,7 +16915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E309"/>
+  <dimension ref="A1:E310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22742,6 +22795,25 @@
       </c>
       <c r="E309" t="n">
         <v>1.45135</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>05/06</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="C310" t="n">
+        <v>-0.205</v>
+      </c>
+      <c r="D310" t="n">
+        <v>2.015</v>
+      </c>
+      <c r="E310" t="n">
+        <v>1.480595</v>
       </c>
     </row>
   </sheetData>
@@ -22755,7 +22827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G289"/>
+  <dimension ref="A1:G290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31147,6 +31219,35 @@
         </is>
       </c>
     </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>05/06</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>1.0583</v>
+      </c>
+      <c r="C290" t="n">
+        <v>3.105</v>
+      </c>
+      <c r="D290" t="n">
+        <v>-2.0467</v>
+      </c>
+      <c r="E290" t="n">
+        <v>0.940754</v>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 煤炭, 钢铁</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 计算机</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update am 24/25 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M310"/>
+  <dimension ref="A1:M311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10990,6 +10990,40 @@
       </c>
       <c r="M310" t="n">
         <v>1.209428</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>05/07</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>-2.9332</v>
+      </c>
+      <c r="D311" t="n">
+        <v>-2.9332</v>
+      </c>
+      <c r="E311" t="n">
+        <v>0.558074</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0.8957000000000001</v>
+      </c>
+      <c r="H311" t="n">
+        <v>0.8957000000000001</v>
+      </c>
+      <c r="I311" t="n">
+        <v>1.107661</v>
+      </c>
+      <c r="J311" t="n">
+        <v>1.4505</v>
+      </c>
+      <c r="L311" t="n">
+        <v>1.4505</v>
+      </c>
+      <c r="M311" t="n">
+        <v>1.22697</v>
       </c>
     </row>
   </sheetData>
@@ -11003,7 +11037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E310"/>
+  <dimension ref="A1:E311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16902,6 +16936,25 @@
       </c>
       <c r="E310" t="n">
         <v>1.781223</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>05/07</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>1.453</v>
+      </c>
+      <c r="C311" t="n">
+        <v>1.3242</v>
+      </c>
+      <c r="D311" t="n">
+        <v>1.3886</v>
+      </c>
+      <c r="E311" t="n">
+        <v>1.805957</v>
       </c>
     </row>
   </sheetData>
@@ -16915,7 +16968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E310"/>
+  <dimension ref="A1:E311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22814,6 +22867,25 @@
       </c>
       <c r="E310" t="n">
         <v>1.480595</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>05/07</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>-1.5467</v>
+      </c>
+      <c r="C311" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="D311" t="n">
+        <v>-1.6517</v>
+      </c>
+      <c r="E311" t="n">
+        <v>1.45614</v>
       </c>
     </row>
   </sheetData>
@@ -22827,7 +22899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G290"/>
+  <dimension ref="A1:G291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31248,6 +31320,35 @@
         </is>
       </c>
     </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>05/07</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>0.0283</v>
+      </c>
+      <c r="C291" t="n">
+        <v>2.0083</v>
+      </c>
+      <c r="D291" t="n">
+        <v>-1.98</v>
+      </c>
+      <c r="E291" t="n">
+        <v>0.922127</v>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 纺织服饰, 煤炭, 钢铁</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 计算机</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update am 20/25 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M311"/>
+  <dimension ref="A1:M312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11024,6 +11024,40 @@
       </c>
       <c r="M311" t="n">
         <v>1.22697</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>05/08</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>1.9514</v>
+      </c>
+      <c r="D312" t="n">
+        <v>1.9514</v>
+      </c>
+      <c r="E312" t="n">
+        <v>0.568964</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0.6797</v>
+      </c>
+      <c r="H312" t="n">
+        <v>0.6797</v>
+      </c>
+      <c r="I312" t="n">
+        <v>1.11519</v>
+      </c>
+      <c r="J312" t="n">
+        <v>1.5809</v>
+      </c>
+      <c r="L312" t="n">
+        <v>1.5809</v>
+      </c>
+      <c r="M312" t="n">
+        <v>1.246367</v>
       </c>
     </row>
   </sheetData>
@@ -11037,7 +11071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E311"/>
+  <dimension ref="A1:E312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16955,6 +16989,25 @@
       </c>
       <c r="E311" t="n">
         <v>1.805957</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>05/08</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>-0.9634</v>
+      </c>
+      <c r="C312" t="n">
+        <v>-2.2888</v>
+      </c>
+      <c r="D312" t="n">
+        <v>-1.6261</v>
+      </c>
+      <c r="E312" t="n">
+        <v>1.77659</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update am 21/25 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M312"/>
+  <dimension ref="A1:M313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11058,6 +11058,40 @@
       </c>
       <c r="M312" t="n">
         <v>1.246367</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026/05/11</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>-4.3731</v>
+      </c>
+      <c r="D313" t="n">
+        <v>-4.3731</v>
+      </c>
+      <c r="E313" t="n">
+        <v>0.544083</v>
+      </c>
+      <c r="F313" t="n">
+        <v>-0.2302</v>
+      </c>
+      <c r="H313" t="n">
+        <v>-0.2302</v>
+      </c>
+      <c r="I313" t="n">
+        <v>1.112622</v>
+      </c>
+      <c r="J313" t="n">
+        <v>-0.5006</v>
+      </c>
+      <c r="L313" t="n">
+        <v>-0.5006</v>
+      </c>
+      <c r="M313" t="n">
+        <v>1.240128</v>
       </c>
     </row>
   </sheetData>
@@ -11071,7 +11105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E312"/>
+  <dimension ref="A1:E313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17008,6 +17042,25 @@
       </c>
       <c r="E312" t="n">
         <v>1.77659</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026/05/11</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>3.4995</v>
+      </c>
+      <c r="C313" t="n">
+        <v>4.6469</v>
+      </c>
+      <c r="D313" t="n">
+        <v>4.0732</v>
+      </c>
+      <c r="E313" t="n">
+        <v>1.848954</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update close 23/25 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M321"/>
+  <dimension ref="A1:M322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11364,6 +11364,40 @@
       </c>
       <c r="M321" t="n">
         <v>1.228841</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>-1.6793</v>
+      </c>
+      <c r="D322" t="n">
+        <v>-1.6793</v>
+      </c>
+      <c r="E322" t="n">
+        <v>0.497479</v>
+      </c>
+      <c r="F322" t="n">
+        <v>-1.0597</v>
+      </c>
+      <c r="H322" t="n">
+        <v>-1.0597</v>
+      </c>
+      <c r="I322" t="n">
+        <v>0.966569</v>
+      </c>
+      <c r="J322" t="n">
+        <v>1.3364</v>
+      </c>
+      <c r="L322" t="n">
+        <v>1.3364</v>
+      </c>
+      <c r="M322" t="n">
+        <v>1.245263</v>
       </c>
     </row>
   </sheetData>
@@ -11377,7 +11411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E321"/>
+  <dimension ref="A1:E322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17485,6 +17519,25 @@
       </c>
       <c r="E321" t="n">
         <v>1.851187</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>2.8389</v>
+      </c>
+      <c r="C322" t="n">
+        <v>1.5076</v>
+      </c>
+      <c r="D322" t="n">
+        <v>2.1733</v>
+      </c>
+      <c r="E322" t="n">
+        <v>1.891418</v>
       </c>
     </row>
   </sheetData>
@@ -17498,7 +17551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E320"/>
+  <dimension ref="A1:E321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23587,6 +23640,25 @@
       </c>
       <c r="E320" t="n">
         <v>1.425334</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026/05/21</t>
+        </is>
+      </c>
+      <c r="B321" t="n">
+        <v>-2.4367</v>
+      </c>
+      <c r="C321" t="n">
+        <v>-0.64</v>
+      </c>
+      <c r="D321" t="n">
+        <v>-1.7967</v>
+      </c>
+      <c r="E321" t="n">
+        <v>1.399725</v>
       </c>
     </row>
   </sheetData>
@@ -23600,7 +23672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G300"/>
+  <dimension ref="A1:G301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32311,6 +32383,35 @@
         </is>
       </c>
     </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026/05/21</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>-2.7083</v>
+      </c>
+      <c r="C301" t="n">
+        <v>-3.405</v>
+      </c>
+      <c r="D301" t="n">
+        <v>0.6967</v>
+      </c>
+      <c r="E301" t="n">
+        <v>0.86471</v>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 钢铁, 煤炭, 纺织服饰</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 计算机</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update close 24/25 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M322"/>
+  <dimension ref="A1:M323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11398,6 +11398,40 @@
       </c>
       <c r="M322" t="n">
         <v>1.245263</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026/05/25</t>
+        </is>
+      </c>
+      <c r="B323" t="n">
+        <v>-5.3897</v>
+      </c>
+      <c r="D323" t="n">
+        <v>-5.3897</v>
+      </c>
+      <c r="E323" t="n">
+        <v>0.470666</v>
+      </c>
+      <c r="F323" t="n">
+        <v>-2.5827</v>
+      </c>
+      <c r="H323" t="n">
+        <v>-2.5827</v>
+      </c>
+      <c r="I323" t="n">
+        <v>0.9416060000000001</v>
+      </c>
+      <c r="J323" t="n">
+        <v>-1.298</v>
+      </c>
+      <c r="L323" t="n">
+        <v>-1.298</v>
+      </c>
+      <c r="M323" t="n">
+        <v>1.2291</v>
       </c>
     </row>
   </sheetData>
@@ -11411,7 +11445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E322"/>
+  <dimension ref="A1:E323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17538,6 +17572,25 @@
       </c>
       <c r="E322" t="n">
         <v>1.891418</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026/05/25</t>
+        </is>
+      </c>
+      <c r="B323" t="n">
+        <v>2.0987</v>
+      </c>
+      <c r="C323" t="n">
+        <v>5.8782</v>
+      </c>
+      <c r="D323" t="n">
+        <v>3.9884</v>
+      </c>
+      <c r="E323" t="n">
+        <v>1.966856</v>
       </c>
     </row>
   </sheetData>
@@ -17551,7 +17604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E321"/>
+  <dimension ref="A1:E322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23659,6 +23712,25 @@
       </c>
       <c r="E321" t="n">
         <v>1.399725</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>1.2767</v>
+      </c>
+      <c r="C322" t="n">
+        <v>-0.905</v>
+      </c>
+      <c r="D322" t="n">
+        <v>2.1817</v>
+      </c>
+      <c r="E322" t="n">
+        <v>1.430263</v>
       </c>
     </row>
   </sheetData>
@@ -23672,7 +23744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G301"/>
+  <dimension ref="A1:G302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32412,6 +32484,35 @@
         </is>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026/05/22</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C302" t="n">
+        <v>2.9783</v>
+      </c>
+      <c r="D302" t="n">
+        <v>-1.8083</v>
+      </c>
+      <c r="E302" t="n">
+        <v>0.849073</v>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>美容护理, 综合, 社会服务, 钢铁, 煤炭, 纺织服饰</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>电子, 电力设备, 通信, 机械设备, 有色金属, 计算机</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: update late_only 7/7 modules
</commit_message>
<xml_diff>
--- a/size_spread/style_spread.xlsx
+++ b/size_spread/style_spread.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M332"/>
+  <dimension ref="A1:M331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11704,40 +11704,6 @@
       </c>
       <c r="M331" t="n">
         <v>1.161674</v>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="inlineStr">
-        <is>
-          <t>2026/06/05</t>
-        </is>
-      </c>
-      <c r="B332" t="n">
-        <v>4.0529</v>
-      </c>
-      <c r="D332" t="n">
-        <v>4.0529</v>
-      </c>
-      <c r="E332" t="n">
-        <v>0.539994</v>
-      </c>
-      <c r="F332" t="n">
-        <v>1.7547</v>
-      </c>
-      <c r="H332" t="n">
-        <v>1.7547</v>
-      </c>
-      <c r="I332" t="n">
-        <v>0.917184</v>
-      </c>
-      <c r="J332" t="n">
-        <v>1.914</v>
-      </c>
-      <c r="L332" t="n">
-        <v>1.914</v>
-      </c>
-      <c r="M332" t="n">
-        <v>1.183909</v>
       </c>
     </row>
   </sheetData>
@@ -11751,7 +11717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E344"/>
+  <dimension ref="A1:E343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18277,25 +18243,6 @@
       </c>
       <c r="E343" t="n">
         <v>1.695853</v>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="inlineStr">
-        <is>
-          <t>2026/06/05</t>
-        </is>
-      </c>
-      <c r="B344" t="n">
-        <v>-3.2026</v>
-      </c>
-      <c r="C344" t="n">
-        <v>-4.0119</v>
-      </c>
-      <c r="D344" t="n">
-        <v>-3.6072</v>
-      </c>
-      <c r="E344" t="n">
-        <v>1.700741</v>
       </c>
     </row>
   </sheetData>

</xml_diff>